<commit_message>
Working through space heating
</commit_message>
<xml_diff>
--- a/[deprecated]/Residential/Ontario/Residential space heating existing capacity.xlsx
+++ b/[deprecated]/Residential/Ontario/Residential space heating existing capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/buildings_sector/[deprecated]/Residential/Ontario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="14_{0D8085FA-641D-4293-8C89-BFDEC87C70DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DA70AA9-E3BD-4315-AA43-20A08E2FB8ED}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="14_{0D8085FA-641D-4293-8C89-BFDEC87C70DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9FF4285-4DF8-4E2F-B708-E19E5A6976B9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,6 +19,7 @@
     <sheet name="secondary energy" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="77">
   <si>
     <t>Residential Sector</t>
   </si>
@@ -371,9 +372,6 @@
     <t>Efficiency</t>
   </si>
   <si>
-    <t>Annual CF</t>
-  </si>
-  <si>
     <t>Assume an arbitrary 1000 PJ/Munityr unit capacity and use this to calculate annual capacity factor which defines actual energy output per unit</t>
   </si>
   <si>
@@ -383,35 +381,30 @@
     <t>exs cap Munits</t>
   </si>
   <si>
-    <t>ann sec energy PJ</t>
-  </si>
-  <si>
-    <t>Arb. c2a PJ/Munityr</t>
-  </si>
-  <si>
     <t>annual act PJ/Munit</t>
   </si>
   <si>
     <t>est c2a PJ/Munityr</t>
   </si>
   <si>
-    <t>ACF</t>
+    <t>DEMAND</t>
   </si>
   <si>
-    <t>DEMAND</t>
+    <t>ann dem PJ</t>
+  </si>
+  <si>
+    <t>annual cap fac</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
-    <numFmt numFmtId="168" formatCode="0.000%"/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -553,7 +546,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -637,8 +630,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="167" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1267,660 +1258,539 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.5703125" customWidth="1"/>
     <col min="2" max="2" width="35.5703125" style="20" customWidth="1"/>
     <col min="3" max="5" width="17.5703125" style="20" customWidth="1"/>
-    <col min="6" max="8" width="22" style="20" customWidth="1"/>
-    <col min="9" max="9" width="19.7109375" customWidth="1"/>
-    <col min="10" max="10" width="25" customWidth="1"/>
-    <col min="11" max="11" width="14.42578125" customWidth="1"/>
-    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22" style="20" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C1" s="35">
         <v>2020</v>
       </c>
       <c r="D1" s="35"/>
       <c r="E1" s="35"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
         <v>52</v>
       </c>
       <c r="B2" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="49" t="s">
+      <c r="C2" s="47" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="49" t="s">
-        <v>68</v>
-      </c>
-      <c r="E2" s="40" t="s">
+      <c r="G2" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="H2" s="44" t="s">
         <v>73</v>
       </c>
-      <c r="F2" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="G2" s="42" t="s">
-        <v>74</v>
-      </c>
-      <c r="H2" s="42" t="s">
-        <v>69</v>
-      </c>
-      <c r="I2" s="42" t="s">
-        <v>71</v>
-      </c>
-      <c r="J2" s="46" t="s">
+      <c r="I2" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="K2" s="46" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="46">
+      <c r="C3" s="44">
         <f>stock!W28/1000</f>
         <v>0</v>
       </c>
-      <c r="D3" s="50">
+      <c r="D3" s="48">
         <f>efficiency!W14/100</f>
         <v>0.6</v>
       </c>
       <c r="E3" s="20">
-        <f>'secondary energy'!W15</f>
-        <v>0</v>
-      </c>
-      <c r="F3" s="20" t="e">
-        <f>D3*E3/C3</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G3" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H3" s="44" t="e">
-        <f>F3/G3</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I3" s="20"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="48"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <f>'secondary energy'!W15*D3</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="20"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="46"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="46">
+      <c r="C4" s="44">
         <f>stock!W29/1000</f>
         <v>0.13224799999999998</v>
       </c>
-      <c r="D4" s="50">
+      <c r="D4" s="48">
         <f>efficiency!W15/100</f>
         <v>0.78</v>
       </c>
       <c r="E4" s="20">
-        <f>'secondary energy'!W16</f>
-        <v>3.7591169999999998</v>
+        <f>'secondary energy'!W16*D4</f>
+        <v>2.9321112600000001</v>
       </c>
       <c r="F4" s="20">
-        <f t="shared" ref="F4:F17" si="0">D4*E4/C4</f>
+        <f>E4/C4</f>
         <v>22.17130890448249</v>
       </c>
-      <c r="G4" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H4" s="44">
-        <f t="shared" ref="H4:H17" si="1">F4/G4</f>
-        <v>2.217130890448249E-2</v>
-      </c>
-      <c r="I4" s="20">
+      <c r="G4" s="20">
         <v>105</v>
       </c>
-      <c r="J4" s="47">
-        <f>I4*$B$21*$B$22*1000000</f>
+      <c r="H4" s="45">
+        <f>G4*$B$21*$B$22*1000000</f>
         <v>970.44014088000029</v>
       </c>
-      <c r="K4" s="48">
-        <f>F4/J4</f>
+      <c r="I4" s="46">
+        <f>F4/H4</f>
         <v>2.2846652740866048E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="46">
+      <c r="C5" s="44">
         <f>stock!W30/1000</f>
         <v>0</v>
       </c>
-      <c r="D5" s="50">
+      <c r="D5" s="48">
         <f>efficiency!W16/100</f>
         <v>0.85</v>
       </c>
       <c r="E5" s="20">
-        <f>'secondary energy'!W17</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="20" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G5" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H5" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I5" s="20"/>
-      <c r="J5" s="47"/>
-      <c r="K5" s="48"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+        <f>'secondary energy'!W17*D5</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="20"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="46"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="44">
         <f>stock!W31/1000</f>
         <v>0</v>
       </c>
-      <c r="D6" s="50">
+      <c r="D6" s="48">
         <f>efficiency!W17/100</f>
         <v>0.62</v>
       </c>
       <c r="E6" s="20">
-        <f>'secondary energy'!W18</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="20" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G6" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H6" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I6" s="20"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="48"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+        <f>'secondary energy'!W18*D6</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="20"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="46"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="46">
+      <c r="C7" s="44">
         <f>stock!W32/1000</f>
         <v>0.72494000000000003</v>
       </c>
-      <c r="D7" s="50">
+      <c r="D7" s="48">
         <f>efficiency!W18/100</f>
         <v>0.8</v>
       </c>
       <c r="E7" s="20">
-        <f>'secondary energy'!W19</f>
-        <v>49.475327</v>
+        <f>'secondary energy'!W19*D7</f>
+        <v>39.5802616</v>
       </c>
       <c r="F7" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="F7:F17" si="0">E7/C7</f>
         <v>54.597982729605206</v>
       </c>
-      <c r="G7" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H7" s="44">
-        <f t="shared" si="1"/>
-        <v>5.4597982729605206E-2</v>
-      </c>
-      <c r="I7" s="20">
+      <c r="G7" s="20">
         <v>80</v>
       </c>
-      <c r="J7" s="47">
-        <f t="shared" ref="J5:J17" si="2">I7*$B$21*$B$22*1000000</f>
+      <c r="H7" s="45">
+        <f t="shared" ref="H7:H17" si="1">G7*$B$21*$B$22*1000000</f>
         <v>739.38296448000017</v>
       </c>
-      <c r="K7" s="48">
-        <f t="shared" ref="K5:K17" si="3">F7/J7</f>
+      <c r="I7" s="46">
+        <f>F7/H7</f>
         <v>7.384263007466417E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="46">
+      <c r="C8" s="44">
         <f>stock!W33/1000</f>
         <v>3.0997629999999998</v>
       </c>
-      <c r="D8" s="50">
+      <c r="D8" s="48">
         <f>efficiency!W19/100</f>
         <v>0.9</v>
       </c>
       <c r="E8" s="20">
-        <f>'secondary energy'!W20</f>
-        <v>184.52887699999999</v>
+        <f>'secondary energy'!W20*D8</f>
+        <v>166.0759893</v>
       </c>
       <c r="F8" s="20">
         <f t="shared" si="0"/>
         <v>53.576995821938652</v>
       </c>
-      <c r="G8" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H8" s="44">
+      <c r="G8" s="20">
+        <v>80</v>
+      </c>
+      <c r="H8" s="45">
         <f t="shared" si="1"/>
-        <v>5.3576995821938651E-2</v>
-      </c>
-      <c r="I8" s="20">
-        <v>80</v>
-      </c>
-      <c r="J8" s="47">
-        <f t="shared" si="2"/>
         <v>739.38296448000017</v>
       </c>
-      <c r="K8" s="48">
-        <f t="shared" si="3"/>
+      <c r="I8" s="46">
+        <f>F8/H8</f>
         <v>7.2461766629447241E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="44">
         <f>stock!W34/1000</f>
         <v>0.98379799999999995</v>
       </c>
-      <c r="D9" s="50">
+      <c r="D9" s="48">
         <f>efficiency!W20/100</f>
         <v>1</v>
       </c>
       <c r="E9" s="20">
-        <f>'secondary energy'!W21</f>
+        <f>'secondary energy'!W21*D9</f>
         <v>34.435597999999999</v>
       </c>
       <c r="F9" s="20">
         <f t="shared" si="0"/>
         <v>35.002711938832974</v>
       </c>
-      <c r="G9" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H9" s="44">
+      <c r="G9" s="20">
+        <v>68</v>
+      </c>
+      <c r="H9" s="45">
         <f t="shared" si="1"/>
-        <v>3.5002711938832975E-2</v>
-      </c>
-      <c r="I9" s="20">
-        <v>68</v>
-      </c>
-      <c r="J9" s="47">
-        <f t="shared" si="2"/>
         <v>628.47551980800006</v>
       </c>
-      <c r="K9" s="48">
-        <f t="shared" si="3"/>
+      <c r="I9" s="46">
+        <f>F9/H9</f>
         <v>5.5694630634978974E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="46">
+      <c r="C10" s="44">
         <f>stock!W35/1000</f>
         <v>0.39461900000000005</v>
       </c>
-      <c r="D10" s="50">
+      <c r="D10" s="48">
         <f>efficiency!W21/100</f>
         <v>1.9</v>
       </c>
       <c r="E10" s="20">
-        <f>'secondary energy'!W22</f>
-        <v>9.7901030000000002</v>
+        <f>'secondary energy'!W22*D10</f>
+        <v>18.601195699999998</v>
       </c>
       <c r="F10" s="20">
         <f t="shared" si="0"/>
         <v>47.137101102582477</v>
       </c>
-      <c r="G10" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H10" s="44">
+      <c r="G10" s="20">
+        <v>36</v>
+      </c>
+      <c r="H10" s="45">
         <f t="shared" si="1"/>
-        <v>4.7137101102582478E-2</v>
-      </c>
-      <c r="I10" s="20">
-        <v>36</v>
-      </c>
-      <c r="J10" s="47">
-        <f t="shared" si="2"/>
         <v>332.72233401600005</v>
       </c>
-      <c r="K10" s="48">
-        <f t="shared" si="3"/>
+      <c r="I10" s="46">
+        <f>F10/H10</f>
         <v>0.14167098593482377</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>50</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="46">
+      <c r="C11" s="44">
         <f>stock!W36/1000</f>
         <v>0.18088699999999999</v>
       </c>
-      <c r="D11" s="50">
+      <c r="D11" s="48">
         <f>efficiency!W22/100</f>
         <v>0.5</v>
       </c>
       <c r="E11" s="20">
-        <f>'secondary energy'!W23</f>
-        <v>7.9320620000000002</v>
+        <f>'secondary energy'!W23*D11</f>
+        <v>3.9660310000000001</v>
       </c>
       <c r="F11" s="20">
         <f t="shared" si="0"/>
         <v>21.925461752364736</v>
       </c>
-      <c r="G11" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H11" s="44">
+      <c r="G11" s="20">
+        <v>80</v>
+      </c>
+      <c r="H11" s="45">
         <f t="shared" si="1"/>
-        <v>2.1925461752364737E-2</v>
-      </c>
-      <c r="I11" s="20">
-        <v>80</v>
-      </c>
-      <c r="J11" s="47">
-        <f t="shared" si="2"/>
         <v>739.38296448000017</v>
       </c>
-      <c r="K11" s="48">
-        <f t="shared" si="3"/>
+      <c r="I11" s="46">
+        <f>F11/H11</f>
         <v>2.9653728589466043E-2</v>
       </c>
-      <c r="L11" s="39"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J11" s="39"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
         <v>14</v>
       </c>
       <c r="B12" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="46">
+      <c r="C12" s="44">
         <f>stock!W37/1000</f>
         <v>2.7367000000000002E-2</v>
       </c>
-      <c r="D12" s="50">
+      <c r="D12" s="48">
         <f>efficiency!W23/100</f>
         <v>0.5</v>
       </c>
       <c r="E12" s="20">
-        <f>'secondary energy'!W24</f>
-        <v>1.468934</v>
+        <f>'secondary energy'!W24*D12</f>
+        <v>0.73446699999999998</v>
       </c>
       <c r="F12" s="20">
         <f t="shared" si="0"/>
         <v>26.837687726093467</v>
       </c>
-      <c r="G12" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H12" s="44">
+      <c r="G12" s="20">
+        <v>50</v>
+      </c>
+      <c r="H12" s="45">
         <f t="shared" si="1"/>
-        <v>2.6837687726093466E-2</v>
-      </c>
-      <c r="I12" s="20">
-        <v>50</v>
-      </c>
-      <c r="J12" s="47">
-        <f t="shared" si="2"/>
         <v>462.11435280000006</v>
       </c>
-      <c r="K12" s="48">
-        <f t="shared" si="3"/>
+      <c r="I12" s="46">
+        <f>F12/H12</f>
         <v>5.807585841790254E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="45" t="s">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="46">
+      <c r="C13" s="44">
         <f>stock!W38/1000</f>
         <v>0</v>
       </c>
-      <c r="D13" s="50"/>
-      <c r="F13" s="20" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G13" s="42"/>
-      <c r="H13" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I13" s="20"/>
-      <c r="J13" s="47"/>
-      <c r="K13" s="48"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D13" s="48"/>
+      <c r="E13" s="20">
+        <f>'secondary energy'!W25*D13</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="20"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="46"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
         <v>44</v>
       </c>
       <c r="B14" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="46">
+      <c r="C14" s="44">
         <f>stock!W39/1000</f>
         <v>0.124442</v>
       </c>
-      <c r="D14" s="50">
+      <c r="D14" s="48">
         <f>efficiency!W27/100</f>
         <v>0.5</v>
       </c>
       <c r="E14" s="20">
-        <f>'secondary energy'!W26</f>
-        <v>14.379021</v>
+        <f>'secondary energy'!W26*D14</f>
+        <v>7.1895104999999999</v>
       </c>
       <c r="F14" s="20">
         <f t="shared" si="0"/>
         <v>57.77398707831761</v>
       </c>
-      <c r="G14" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H14" s="44">
+      <c r="G14" s="20">
+        <v>50</v>
+      </c>
+      <c r="H14" s="45">
         <f t="shared" si="1"/>
-        <v>5.7773987078317608E-2</v>
-      </c>
-      <c r="I14" s="20">
-        <v>50</v>
-      </c>
-      <c r="J14" s="47">
-        <f t="shared" si="2"/>
         <v>462.11435280000006</v>
       </c>
-      <c r="K14" s="48">
-        <f t="shared" si="3"/>
+      <c r="I14" s="46">
+        <f>F14/H14</f>
         <v>0.1250209752808128</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="20" t="s">
         <v>47</v>
       </c>
       <c r="B15" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C15" s="46">
+      <c r="C15" s="44">
         <f>stock!W40/1000</f>
         <v>0.11401</v>
       </c>
-      <c r="D15" s="50">
+      <c r="D15" s="48">
         <f>efficiency!W30/100</f>
         <v>0.78</v>
       </c>
       <c r="E15" s="20">
-        <f>'secondary energy'!W27</f>
-        <v>5.7887409999999999</v>
+        <f>'secondary energy'!W27*D15</f>
+        <v>4.5152179800000001</v>
       </c>
       <c r="F15" s="20">
         <f t="shared" si="0"/>
         <v>39.60370125427594</v>
       </c>
-      <c r="G15" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H15" s="44">
+      <c r="G15" s="20">
+        <v>105</v>
+      </c>
+      <c r="H15" s="45">
         <f t="shared" si="1"/>
-        <v>3.9603701254275939E-2</v>
-      </c>
-      <c r="I15" s="20">
-        <v>105</v>
-      </c>
-      <c r="J15" s="47">
-        <f t="shared" si="2"/>
         <v>970.44014088000029</v>
       </c>
-      <c r="K15" s="48">
-        <f t="shared" si="3"/>
+      <c r="I15" s="46">
+        <f>F15/H15</f>
         <v>4.0810040296110475E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="s">
         <v>45</v>
       </c>
       <c r="B16" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="46">
+      <c r="C16" s="44">
         <f>stock!W41/1000</f>
         <v>3.3182000000000003E-2</v>
       </c>
-      <c r="D16" s="50">
+      <c r="D16" s="48">
         <f>efficiency!W35/100</f>
         <v>0.8</v>
       </c>
       <c r="E16" s="20">
-        <f>'secondary energy'!W28</f>
-        <v>2.3603200000000002</v>
+        <f>'secondary energy'!W28*D16</f>
+        <v>1.8882560000000002</v>
       </c>
       <c r="F16" s="20">
         <f t="shared" si="0"/>
         <v>56.906033391597852</v>
       </c>
-      <c r="G16" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H16" s="44">
+      <c r="G16" s="20">
+        <v>80</v>
+      </c>
+      <c r="H16" s="45">
         <f t="shared" si="1"/>
-        <v>5.6906033391597853E-2</v>
-      </c>
-      <c r="I16" s="20">
-        <v>80</v>
-      </c>
-      <c r="J16" s="47">
-        <f t="shared" si="2"/>
         <v>739.38296448000017</v>
       </c>
-      <c r="K16" s="48">
-        <f t="shared" si="3"/>
+      <c r="I16" s="46">
+        <f>F16/H16</f>
         <v>7.6964220336911915E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="20" t="s">
         <v>46</v>
       </c>
       <c r="B17" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="46">
+      <c r="C17" s="44">
         <f>stock!W42/1000</f>
         <v>2.0537E-2</v>
       </c>
-      <c r="D17" s="50">
+      <c r="D17" s="48">
         <f>efficiency!W39/100</f>
         <v>0.78</v>
       </c>
       <c r="E17" s="20">
-        <f>'secondary energy'!W29</f>
-        <v>0.71361300000000005</v>
+        <f>'secondary energy'!W29*D17</f>
+        <v>0.55661814000000009</v>
       </c>
       <c r="F17" s="20">
         <f t="shared" si="0"/>
         <v>27.103186443979165</v>
       </c>
-      <c r="G17" s="42">
-        <v>1000</v>
-      </c>
-      <c r="H17" s="44">
+      <c r="G17">
+        <v>105</v>
+      </c>
+      <c r="H17" s="45">
         <f t="shared" si="1"/>
-        <v>2.7103186443979164E-2</v>
-      </c>
-      <c r="I17">
-        <v>105</v>
-      </c>
-      <c r="J17" s="47">
-        <f t="shared" si="2"/>
         <v>970.44014088000029</v>
       </c>
-      <c r="K17" s="48">
-        <f t="shared" si="3"/>
+      <c r="I17" s="46">
+        <f>F17/H17</f>
         <v>2.7928756553085132E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="20"/>
     </row>
-    <row r="19" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
         <v>66</v>
       </c>
       <c r="C19" s="20">
         <v>1</v>
       </c>
-      <c r="E19" s="47">
+      <c r="E19" s="45">
         <f>SUM(E3:E17)</f>
-        <v>314.63171299999999</v>
-      </c>
-      <c r="F19" s="46" t="s">
-        <v>78</v>
-      </c>
-      <c r="J19" s="41"/>
-    </row>
-    <row r="20" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+        <v>280.47525647999998</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="H19" s="41"/>
+    </row>
+    <row r="20" spans="1:9" s="20" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
         <v>48</v>
       </c>
@@ -1932,11 +1802,9 @@
         <v>49</v>
       </c>
       <c r="F21" s="23"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="40"/>
-      <c r="J21" s="41"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H21" s="41"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="s">
         <v>51</v>
       </c>
@@ -1947,34 +1815,33 @@
       <c r="C22" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="H22" s="43"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J27" s="40"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J28" s="40"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J29" s="40"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H27" s="40"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H28" s="40"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H29" s="40"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="20"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="20"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="20"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Finished space heating and generic
</commit_message>
<xml_diff>
--- a/[deprecated]/Residential/Ontario/Residential space heating existing capacity.xlsx
+++ b/[deprecated]/Residential/Ontario/Residential space heating existing capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/buildings_sector/[deprecated]/Residential/Ontario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="14_{0D8085FA-641D-4293-8C89-BFDEC87C70DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9FF4285-4DF8-4E2F-B708-E19E5A6976B9}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="14_{0D8085FA-641D-4293-8C89-BFDEC87C70DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3A52AA0-5F1E-4A84-A5A3-197F716BBB61}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,6 @@
     <sheet name="secondary energy" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="78">
   <si>
     <t>Residential Sector</t>
   </si>
@@ -381,19 +380,22 @@
     <t>exs cap Munits</t>
   </si>
   <si>
-    <t>annual act PJ/Munit</t>
-  </si>
-  <si>
     <t>est c2a PJ/Munityr</t>
   </si>
   <si>
     <t>DEMAND</t>
   </si>
   <si>
-    <t>ann dem PJ</t>
+    <t>annual cap fac</t>
   </si>
   <si>
-    <t>annual cap fac</t>
+    <t>arb. C2a PJ/Munityr</t>
+  </si>
+  <si>
+    <t>ann activity PJ</t>
+  </si>
+  <si>
+    <t>ann unit act PJ/Munityr</t>
   </si>
 </sst>
 </file>
@@ -546,7 +548,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -636,6 +638,7 @@
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1258,7 +1261,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.5703125" customWidth="1"/>
@@ -1267,18 +1270,19 @@
     <col min="6" max="6" width="22" style="20" customWidth="1"/>
     <col min="7" max="7" width="19.7109375" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" customWidth="1"/>
-    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25" style="20" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" customWidth="1"/>
+    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C1" s="35">
         <v>2020</v>
       </c>
       <c r="D1" s="35"/>
       <c r="E1" s="35"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
         <v>52</v>
       </c>
@@ -1292,27 +1296,30 @@
         <v>68</v>
       </c>
       <c r="E2" s="40" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G2" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="44" t="s">
-        <v>73</v>
+      <c r="H2" s="42" t="s">
+        <v>72</v>
       </c>
       <c r="I2" s="44" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="J2" s="44" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="44">
-        <f>stock!W28/1000</f>
+        <f>stock!W28</f>
         <v>0</v>
       </c>
       <c r="D3" s="48">
@@ -1324,10 +1331,11 @@
         <v>0</v>
       </c>
       <c r="G3" s="20"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="46"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H3" s="49"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="46"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>6</v>
       </c>
@@ -1353,16 +1361,19 @@
       <c r="G4" s="20">
         <v>105</v>
       </c>
-      <c r="H4" s="45">
+      <c r="H4" s="49">
         <f>G4*$B$21*$B$22*1000000</f>
         <v>970.44014088000029</v>
       </c>
-      <c r="I4" s="46">
-        <f>F4/H4</f>
-        <v>2.2846652740866048E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I4" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J4" s="46">
+        <f>F4/I4</f>
+        <v>2.217130890448249E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
         <v>7</v>
       </c>
@@ -1379,10 +1390,11 @@
         <v>0</v>
       </c>
       <c r="G5" s="20"/>
-      <c r="H5" s="45"/>
-      <c r="I5" s="46"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H5" s="49"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="46"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
         <v>8</v>
       </c>
@@ -1399,10 +1411,11 @@
         <v>0</v>
       </c>
       <c r="G6" s="20"/>
-      <c r="H6" s="45"/>
-      <c r="I6" s="46"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H6" s="49"/>
+      <c r="I6" s="45"/>
+      <c r="J6" s="46"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
@@ -1428,16 +1441,19 @@
       <c r="G7" s="20">
         <v>80</v>
       </c>
-      <c r="H7" s="45">
+      <c r="H7" s="49">
         <f t="shared" ref="H7:H17" si="1">G7*$B$21*$B$22*1000000</f>
         <v>739.38296448000017</v>
       </c>
-      <c r="I7" s="46">
-        <f>F7/H7</f>
-        <v>7.384263007466417E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I7" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J7" s="46">
+        <f t="shared" ref="J5:J17" si="2">F7/I7</f>
+        <v>5.4597982729605206E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
         <v>10</v>
       </c>
@@ -1463,16 +1479,19 @@
       <c r="G8" s="20">
         <v>80</v>
       </c>
-      <c r="H8" s="45">
+      <c r="H8" s="49">
         <f t="shared" si="1"/>
         <v>739.38296448000017</v>
       </c>
-      <c r="I8" s="46">
-        <f>F8/H8</f>
-        <v>7.2461766629447241E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I8" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J8" s="46">
+        <f t="shared" si="2"/>
+        <v>5.3576995821938651E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
         <v>11</v>
       </c>
@@ -1498,16 +1517,19 @@
       <c r="G9" s="20">
         <v>68</v>
       </c>
-      <c r="H9" s="45">
+      <c r="H9" s="49">
         <f t="shared" si="1"/>
         <v>628.47551980800006</v>
       </c>
-      <c r="I9" s="46">
-        <f>F9/H9</f>
-        <v>5.5694630634978974E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I9" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J9" s="46">
+        <f t="shared" si="2"/>
+        <v>3.5002711938832975E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>12</v>
       </c>
@@ -1533,16 +1555,19 @@
       <c r="G10" s="20">
         <v>36</v>
       </c>
-      <c r="H10" s="45">
+      <c r="H10" s="49">
         <f t="shared" si="1"/>
         <v>332.72233401600005</v>
       </c>
-      <c r="I10" s="46">
-        <f>F10/H10</f>
-        <v>0.14167098593482377</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I10" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J10" s="46">
+        <f t="shared" si="2"/>
+        <v>4.7137101102582478E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>50</v>
       </c>
@@ -1568,17 +1593,20 @@
       <c r="G11" s="20">
         <v>80</v>
       </c>
-      <c r="H11" s="45">
+      <c r="H11" s="49">
         <f t="shared" si="1"/>
         <v>739.38296448000017</v>
       </c>
-      <c r="I11" s="46">
-        <f>F11/H11</f>
-        <v>2.9653728589466043E-2</v>
-      </c>
-      <c r="J11" s="39"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I11" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J11" s="46">
+        <f t="shared" si="2"/>
+        <v>2.1925461752364737E-2</v>
+      </c>
+      <c r="K11" s="39"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
         <v>14</v>
       </c>
@@ -1604,16 +1632,19 @@
       <c r="G12" s="20">
         <v>50</v>
       </c>
-      <c r="H12" s="45">
+      <c r="H12" s="49">
         <f t="shared" si="1"/>
         <v>462.11435280000006</v>
       </c>
-      <c r="I12" s="46">
-        <f>F12/H12</f>
-        <v>5.807585841790254E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I12" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J12" s="46">
+        <f t="shared" si="2"/>
+        <v>2.6837687726093466E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="43" t="s">
         <v>15</v>
       </c>
@@ -1627,10 +1658,11 @@
         <v>0</v>
       </c>
       <c r="G13" s="20"/>
-      <c r="H13" s="45"/>
-      <c r="I13" s="46"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H13" s="49"/>
+      <c r="I13" s="45"/>
+      <c r="J13" s="46"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
         <v>44</v>
       </c>
@@ -1656,16 +1688,19 @@
       <c r="G14" s="20">
         <v>50</v>
       </c>
-      <c r="H14" s="45">
+      <c r="H14" s="49">
         <f t="shared" si="1"/>
         <v>462.11435280000006</v>
       </c>
-      <c r="I14" s="46">
-        <f>F14/H14</f>
-        <v>0.1250209752808128</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I14" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J14" s="46">
+        <f t="shared" si="2"/>
+        <v>5.7773987078317608E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="20" t="s">
         <v>47</v>
       </c>
@@ -1691,16 +1726,19 @@
       <c r="G15" s="20">
         <v>105</v>
       </c>
-      <c r="H15" s="45">
+      <c r="H15" s="49">
         <f t="shared" si="1"/>
         <v>970.44014088000029</v>
       </c>
-      <c r="I15" s="46">
-        <f>F15/H15</f>
-        <v>4.0810040296110475E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I15" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J15" s="46">
+        <f t="shared" si="2"/>
+        <v>3.9603701254275939E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="s">
         <v>45</v>
       </c>
@@ -1726,16 +1764,19 @@
       <c r="G16" s="20">
         <v>80</v>
       </c>
-      <c r="H16" s="45">
+      <c r="H16" s="49">
         <f t="shared" si="1"/>
         <v>739.38296448000017</v>
       </c>
-      <c r="I16" s="46">
-        <f>F16/H16</f>
-        <v>7.6964220336911915E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I16" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J16" s="46">
+        <f t="shared" si="2"/>
+        <v>5.6906033391597853E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="20" t="s">
         <v>46</v>
       </c>
@@ -1761,19 +1802,22 @@
       <c r="G17">
         <v>105</v>
       </c>
-      <c r="H17" s="45">
+      <c r="H17" s="49">
         <f t="shared" si="1"/>
         <v>970.44014088000029</v>
       </c>
-      <c r="I17" s="46">
-        <f>F17/H17</f>
-        <v>2.7928756553085132E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I17" s="45">
+        <v>1000</v>
+      </c>
+      <c r="J17" s="46">
+        <f t="shared" si="2"/>
+        <v>2.7103186443979164E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="20"/>
     </row>
-    <row r="19" spans="1:9" s="20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
         <v>66</v>
       </c>
@@ -1785,12 +1829,13 @@
         <v>280.47525647999998</v>
       </c>
       <c r="F19" s="44" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H19" s="41"/>
-    </row>
-    <row r="20" spans="1:9" s="20" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I19" s="41"/>
+    </row>
+    <row r="20" spans="1:10" s="20" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
         <v>48</v>
       </c>
@@ -1803,8 +1848,9 @@
       </c>
       <c r="F21" s="23"/>
       <c r="H21" s="41"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I21" s="41"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="s">
         <v>51</v>
       </c>
@@ -1816,32 +1862,35 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H27" s="40"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I27" s="40"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H28" s="40"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I28" s="40"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H29" s="40"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I29" s="40"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="20"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="20"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="20"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>